<commit_message>
Add freeze panes functionality to Excel export and update raw data files
</commit_message>
<xml_diff>
--- a/data/raw_data.xlsx
+++ b/data/raw_data.xlsx
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ1"/>
+  <dimension ref="A1:AZ23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="3" min="1" max="1"/>
@@ -900,6 +900,2722 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>MND-02</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>DUMMY. Levels = latest old form MND_02.pdf (total 45); MM/YYYY dates invented, onset back-dated to 11/2025. DUMMY. Treatment dates invented. last_assessed = month of the latest old form.</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>11/2025</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr"/>
+      <c r="G2" s="3" t="inlineStr"/>
+      <c r="H2" s="3" t="inlineStr"/>
+      <c r="I2" s="3" t="inlineStr"/>
+      <c r="J2" s="3" t="inlineStr"/>
+      <c r="K2" s="3" t="inlineStr"/>
+      <c r="L2" s="3" t="inlineStr"/>
+      <c r="M2" s="3" t="inlineStr"/>
+      <c r="N2" s="3" t="inlineStr"/>
+      <c r="O2" s="3" t="inlineStr"/>
+      <c r="P2" s="3" t="inlineStr"/>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>12/2025</t>
+        </is>
+      </c>
+      <c r="R2" s="3" t="inlineStr"/>
+      <c r="S2" s="3" t="inlineStr"/>
+      <c r="T2" s="3" t="inlineStr"/>
+      <c r="U2" s="3" t="inlineStr"/>
+      <c r="V2" s="3" t="inlineStr"/>
+      <c r="W2" s="3" t="inlineStr"/>
+      <c r="X2" s="3" t="inlineStr"/>
+      <c r="Y2" s="3" t="inlineStr"/>
+      <c r="Z2" s="3" t="inlineStr"/>
+      <c r="AA2" s="3" t="inlineStr"/>
+      <c r="AB2" s="3" t="inlineStr"/>
+      <c r="AC2" s="3" t="inlineStr"/>
+      <c r="AD2" s="3" t="inlineStr"/>
+      <c r="AE2" s="3" t="inlineStr"/>
+      <c r="AF2" s="3" t="inlineStr"/>
+      <c r="AG2" s="3" t="inlineStr"/>
+      <c r="AH2" s="3" t="inlineStr"/>
+      <c r="AI2" s="3" t="inlineStr"/>
+      <c r="AJ2" s="3" t="inlineStr"/>
+      <c r="AK2" s="3" t="inlineStr">
+        <is>
+          <t>11/2025</t>
+        </is>
+      </c>
+      <c r="AL2" s="3" t="inlineStr"/>
+      <c r="AM2" s="3" t="inlineStr"/>
+      <c r="AN2" s="3" t="inlineStr"/>
+      <c r="AO2" s="3" t="inlineStr"/>
+      <c r="AP2" s="3" t="inlineStr"/>
+      <c r="AQ2" s="3" t="inlineStr"/>
+      <c r="AR2" s="3" t="inlineStr"/>
+      <c r="AS2" s="3" t="inlineStr"/>
+      <c r="AT2" s="3" t="inlineStr"/>
+      <c r="AU2" s="3" t="inlineStr"/>
+      <c r="AV2" s="3" t="inlineStr"/>
+      <c r="AW2" s="3" t="inlineStr"/>
+      <c r="AX2" s="3" t="inlineStr"/>
+      <c r="AY2" s="3" t="inlineStr"/>
+      <c r="AZ2" s="3" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>MND-04</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>DUMMY. Levels = latest old form MND_04.pdf (total 43); MM/YYYY dates invented, onset back-dated to 09/2025. DUMMY. Treatment dates invented. last_assessed = month of the latest old form.</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>09/2025</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr"/>
+      <c r="H3" s="3" t="inlineStr"/>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>11/2025</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr"/>
+      <c r="K3" s="3" t="inlineStr"/>
+      <c r="L3" s="3" t="inlineStr"/>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>10/2025</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr"/>
+      <c r="O3" s="3" t="inlineStr"/>
+      <c r="P3" s="3" t="inlineStr"/>
+      <c r="Q3" s="3" t="inlineStr"/>
+      <c r="R3" s="3" t="inlineStr"/>
+      <c r="S3" s="3" t="inlineStr"/>
+      <c r="T3" s="3" t="inlineStr"/>
+      <c r="U3" s="3" t="inlineStr"/>
+      <c r="V3" s="3" t="inlineStr"/>
+      <c r="W3" s="3" t="inlineStr"/>
+      <c r="X3" s="3" t="inlineStr"/>
+      <c r="Y3" s="3" t="inlineStr"/>
+      <c r="Z3" s="3" t="inlineStr"/>
+      <c r="AA3" s="3" t="inlineStr"/>
+      <c r="AB3" s="3" t="inlineStr"/>
+      <c r="AC3" s="3" t="inlineStr"/>
+      <c r="AD3" s="3" t="inlineStr"/>
+      <c r="AE3" s="3" t="inlineStr"/>
+      <c r="AF3" s="3" t="inlineStr"/>
+      <c r="AG3" s="3" t="inlineStr">
+        <is>
+          <t>11/2025</t>
+        </is>
+      </c>
+      <c r="AH3" s="3" t="inlineStr"/>
+      <c r="AI3" s="3" t="inlineStr"/>
+      <c r="AJ3" s="3" t="inlineStr"/>
+      <c r="AK3" s="3" t="inlineStr">
+        <is>
+          <t>10/2025</t>
+        </is>
+      </c>
+      <c r="AL3" s="3" t="inlineStr"/>
+      <c r="AM3" s="3" t="inlineStr"/>
+      <c r="AN3" s="3" t="inlineStr"/>
+      <c r="AO3" s="3" t="inlineStr"/>
+      <c r="AP3" s="3" t="inlineStr"/>
+      <c r="AQ3" s="3" t="inlineStr"/>
+      <c r="AR3" s="3" t="inlineStr"/>
+      <c r="AS3" s="3" t="inlineStr"/>
+      <c r="AT3" s="3" t="inlineStr"/>
+      <c r="AU3" s="3" t="inlineStr"/>
+      <c r="AV3" s="3" t="inlineStr"/>
+      <c r="AW3" s="3" t="inlineStr"/>
+      <c r="AX3" s="3" t="inlineStr"/>
+      <c r="AY3" s="3" t="inlineStr"/>
+      <c r="AZ3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>MND-05</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>DUMMY. Levels = latest old form MND_05.pdf (total 41); MM/YYYY dates invented, onset back-dated to 07/2025. DUMMY. Treatment dates invented. last_assessed = month of the latest old form.</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>07/2025</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>10/2025</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr"/>
+      <c r="H4" s="3" t="inlineStr"/>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>11/2025</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr"/>
+      <c r="K4" s="3" t="inlineStr"/>
+      <c r="L4" s="3" t="inlineStr"/>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>10/2025</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr"/>
+      <c r="O4" s="3" t="inlineStr"/>
+      <c r="P4" s="3" t="inlineStr"/>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>07/2025</t>
+        </is>
+      </c>
+      <c r="R4" s="3" t="inlineStr"/>
+      <c r="S4" s="3" t="inlineStr"/>
+      <c r="T4" s="3" t="inlineStr"/>
+      <c r="U4" s="3" t="inlineStr">
+        <is>
+          <t>10/2025</t>
+        </is>
+      </c>
+      <c r="V4" s="3" t="inlineStr"/>
+      <c r="W4" s="3" t="inlineStr"/>
+      <c r="X4" s="3" t="inlineStr"/>
+      <c r="Y4" s="3" t="inlineStr">
+        <is>
+          <t>11/2025</t>
+        </is>
+      </c>
+      <c r="Z4" s="3" t="inlineStr"/>
+      <c r="AA4" s="3" t="inlineStr"/>
+      <c r="AB4" s="3" t="inlineStr"/>
+      <c r="AC4" s="3" t="inlineStr"/>
+      <c r="AD4" s="3" t="inlineStr"/>
+      <c r="AE4" s="3" t="inlineStr"/>
+      <c r="AF4" s="3" t="inlineStr"/>
+      <c r="AG4" s="3" t="inlineStr"/>
+      <c r="AH4" s="3" t="inlineStr"/>
+      <c r="AI4" s="3" t="inlineStr"/>
+      <c r="AJ4" s="3" t="inlineStr"/>
+      <c r="AK4" s="3" t="inlineStr"/>
+      <c r="AL4" s="3" t="inlineStr"/>
+      <c r="AM4" s="3" t="inlineStr"/>
+      <c r="AN4" s="3" t="inlineStr"/>
+      <c r="AO4" s="3" t="inlineStr"/>
+      <c r="AP4" s="3" t="inlineStr"/>
+      <c r="AQ4" s="3" t="inlineStr"/>
+      <c r="AR4" s="3" t="inlineStr"/>
+      <c r="AS4" s="3" t="inlineStr"/>
+      <c r="AT4" s="3" t="inlineStr"/>
+      <c r="AU4" s="3" t="inlineStr"/>
+      <c r="AV4" s="3" t="inlineStr"/>
+      <c r="AW4" s="3" t="inlineStr"/>
+      <c r="AX4" s="3" t="inlineStr"/>
+      <c r="AY4" s="3" t="inlineStr"/>
+      <c r="AZ4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>MND-06</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>06/2026</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>DUMMY. Levels = latest old form MND_06.pdf (total 45); MM/YYYY dates invented, onset back-dated to 01/2026. DUMMY. Treatment dates invented. last_assessed = month of the latest old form.</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="3" t="inlineStr"/>
+      <c r="H5" s="3" t="inlineStr"/>
+      <c r="I5" s="3" t="inlineStr"/>
+      <c r="J5" s="3" t="inlineStr"/>
+      <c r="K5" s="3" t="inlineStr"/>
+      <c r="L5" s="3" t="inlineStr"/>
+      <c r="M5" s="3" t="inlineStr"/>
+      <c r="N5" s="3" t="inlineStr"/>
+      <c r="O5" s="3" t="inlineStr"/>
+      <c r="P5" s="3" t="inlineStr"/>
+      <c r="Q5" s="3" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="R5" s="3" t="inlineStr"/>
+      <c r="S5" s="3" t="inlineStr"/>
+      <c r="T5" s="3" t="inlineStr"/>
+      <c r="U5" s="3" t="inlineStr"/>
+      <c r="V5" s="3" t="inlineStr"/>
+      <c r="W5" s="3" t="inlineStr"/>
+      <c r="X5" s="3" t="inlineStr"/>
+      <c r="Y5" s="3" t="inlineStr"/>
+      <c r="Z5" s="3" t="inlineStr"/>
+      <c r="AA5" s="3" t="inlineStr"/>
+      <c r="AB5" s="3" t="inlineStr"/>
+      <c r="AC5" s="3" t="inlineStr"/>
+      <c r="AD5" s="3" t="inlineStr"/>
+      <c r="AE5" s="3" t="inlineStr"/>
+      <c r="AF5" s="3" t="inlineStr"/>
+      <c r="AG5" s="3" t="inlineStr">
+        <is>
+          <t>02/2026</t>
+        </is>
+      </c>
+      <c r="AH5" s="3" t="inlineStr"/>
+      <c r="AI5" s="3" t="inlineStr"/>
+      <c r="AJ5" s="3" t="inlineStr"/>
+      <c r="AK5" s="3" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="AL5" s="3" t="inlineStr"/>
+      <c r="AM5" s="3" t="inlineStr"/>
+      <c r="AN5" s="3" t="inlineStr"/>
+      <c r="AO5" s="3" t="inlineStr"/>
+      <c r="AP5" s="3" t="inlineStr"/>
+      <c r="AQ5" s="3" t="inlineStr"/>
+      <c r="AR5" s="3" t="inlineStr"/>
+      <c r="AS5" s="3" t="inlineStr"/>
+      <c r="AT5" s="3" t="inlineStr"/>
+      <c r="AU5" s="3" t="inlineStr"/>
+      <c r="AV5" s="3" t="inlineStr"/>
+      <c r="AW5" s="3" t="inlineStr"/>
+      <c r="AX5" s="3" t="inlineStr"/>
+      <c r="AY5" s="3" t="inlineStr"/>
+      <c r="AZ5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>MND-07</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>07/2026</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>DUMMY. Levels = latest old form MND_07.pdf (total 25); MM/YYYY dates invented, onset back-dated to 11/2024; old form undated, assessment month assumed 07/2026. DUMMY. Treatment dates invented. last_assessed = month of the latest old form (assumed, old form undated).</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>12/2024</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>05/2025</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr"/>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>09/2025</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr"/>
+      <c r="L6" s="3" t="inlineStr"/>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>11/2024</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>05/2025</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+      <c r="P6" s="3" t="inlineStr">
+        <is>
+          <t>03/2026</t>
+        </is>
+      </c>
+      <c r="Q6" s="3" t="inlineStr"/>
+      <c r="R6" s="3" t="inlineStr"/>
+      <c r="S6" s="3" t="inlineStr"/>
+      <c r="T6" s="3" t="inlineStr"/>
+      <c r="U6" s="3" t="inlineStr"/>
+      <c r="V6" s="3" t="inlineStr"/>
+      <c r="W6" s="3" t="inlineStr"/>
+      <c r="X6" s="3" t="inlineStr"/>
+      <c r="Y6" s="3" t="inlineStr"/>
+      <c r="Z6" s="3" t="inlineStr"/>
+      <c r="AA6" s="3" t="inlineStr"/>
+      <c r="AB6" s="3" t="inlineStr"/>
+      <c r="AC6" s="3" t="inlineStr">
+        <is>
+          <t>12/2024</t>
+        </is>
+      </c>
+      <c r="AD6" s="3" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
+      <c r="AE6" s="3" t="inlineStr">
+        <is>
+          <t>09/2025</t>
+        </is>
+      </c>
+      <c r="AF6" s="3" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="AG6" s="3" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
+      <c r="AH6" s="3" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+      <c r="AI6" s="3" t="inlineStr">
+        <is>
+          <t>03/2026</t>
+        </is>
+      </c>
+      <c r="AJ6" s="3" t="inlineStr"/>
+      <c r="AK6" s="3" t="inlineStr">
+        <is>
+          <t>02/2025</t>
+        </is>
+      </c>
+      <c r="AL6" s="3" t="inlineStr"/>
+      <c r="AM6" s="3" t="inlineStr"/>
+      <c r="AN6" s="3" t="inlineStr"/>
+      <c r="AO6" s="3" t="inlineStr">
+        <is>
+          <t>02/2025</t>
+        </is>
+      </c>
+      <c r="AP6" s="3" t="inlineStr">
+        <is>
+          <t>07/2025</t>
+        </is>
+      </c>
+      <c r="AQ6" s="3" t="inlineStr">
+        <is>
+          <t>03/2026</t>
+        </is>
+      </c>
+      <c r="AR6" s="3" t="inlineStr"/>
+      <c r="AS6" s="3" t="inlineStr"/>
+      <c r="AT6" s="3" t="inlineStr"/>
+      <c r="AU6" s="3" t="inlineStr"/>
+      <c r="AV6" s="3" t="inlineStr"/>
+      <c r="AW6" s="3" t="inlineStr">
+        <is>
+          <t>12/2024</t>
+        </is>
+      </c>
+      <c r="AX6" s="3" t="inlineStr">
+        <is>
+          <t>06/2025</t>
+        </is>
+      </c>
+      <c r="AY6" s="3" t="inlineStr">
+        <is>
+          <t>11/2025</t>
+        </is>
+      </c>
+      <c r="AZ6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>MND-08</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>08/2026</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>DUMMY. Levels = latest old form MND_08_11Aug2026.pdf (total 18); old forms in order: MND_08_27Jan2026.pdf (19), MND_08_10Mar2026.pdf (22), MND_08_11Aug2026.pdf (18); MM/YYYY dates invented, onset back-dated to 01/2024; earlier old form scored lower, latest level kept: q6 0→1, q7 1→2, q11 2→4, q12 1→2. DUMMY. Treatment dates invented. last_assessed = month of the latest old form.</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>02/2026</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>02/2026</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr"/>
+      <c r="H7" s="3" t="inlineStr"/>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>04/2024</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>02/2025</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr"/>
+      <c r="L7" s="3" t="inlineStr"/>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>05/2025</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="inlineStr"/>
+      <c r="O7" s="3" t="inlineStr"/>
+      <c r="P7" s="3" t="inlineStr"/>
+      <c r="Q7" s="3" t="inlineStr">
+        <is>
+          <t>01/2024</t>
+        </is>
+      </c>
+      <c r="R7" s="3" t="inlineStr">
+        <is>
+          <t>07/2024</t>
+        </is>
+      </c>
+      <c r="S7" s="3" t="inlineStr">
+        <is>
+          <t>02/2025</t>
+        </is>
+      </c>
+      <c r="T7" s="3" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+      <c r="U7" s="3" t="inlineStr">
+        <is>
+          <t>05/2024</t>
+        </is>
+      </c>
+      <c r="V7" s="3" t="inlineStr">
+        <is>
+          <t>09/2024</t>
+        </is>
+      </c>
+      <c r="W7" s="3" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
+      <c r="X7" s="3" t="inlineStr">
+        <is>
+          <t>07/2025</t>
+        </is>
+      </c>
+      <c r="Y7" s="3" t="inlineStr">
+        <is>
+          <t>02/2024</t>
+        </is>
+      </c>
+      <c r="Z7" s="3" t="inlineStr">
+        <is>
+          <t>10/2024</t>
+        </is>
+      </c>
+      <c r="AA7" s="3" t="inlineStr">
+        <is>
+          <t>07/2025</t>
+        </is>
+      </c>
+      <c r="AB7" s="3" t="inlineStr"/>
+      <c r="AC7" s="3" t="inlineStr">
+        <is>
+          <t>03/2024</t>
+        </is>
+      </c>
+      <c r="AD7" s="3" t="inlineStr">
+        <is>
+          <t>05/2025</t>
+        </is>
+      </c>
+      <c r="AE7" s="3" t="inlineStr"/>
+      <c r="AF7" s="3" t="inlineStr"/>
+      <c r="AG7" s="3" t="inlineStr">
+        <is>
+          <t>05/2024</t>
+        </is>
+      </c>
+      <c r="AH7" s="3" t="inlineStr">
+        <is>
+          <t>11/2024</t>
+        </is>
+      </c>
+      <c r="AI7" s="3" t="inlineStr">
+        <is>
+          <t>07/2025</t>
+        </is>
+      </c>
+      <c r="AJ7" s="3" t="inlineStr"/>
+      <c r="AK7" s="3" t="inlineStr">
+        <is>
+          <t>02/2024</t>
+        </is>
+      </c>
+      <c r="AL7" s="3" t="inlineStr">
+        <is>
+          <t>06/2024</t>
+        </is>
+      </c>
+      <c r="AM7" s="3" t="inlineStr">
+        <is>
+          <t>02/2025</t>
+        </is>
+      </c>
+      <c r="AN7" s="3" t="inlineStr">
+        <is>
+          <t>07/2025</t>
+        </is>
+      </c>
+      <c r="AO7" s="3" t="inlineStr">
+        <is>
+          <t>08/2024</t>
+        </is>
+      </c>
+      <c r="AP7" s="3" t="inlineStr">
+        <is>
+          <t>02/2025</t>
+        </is>
+      </c>
+      <c r="AQ7" s="3" t="inlineStr">
+        <is>
+          <t>07/2025</t>
+        </is>
+      </c>
+      <c r="AR7" s="3" t="inlineStr"/>
+      <c r="AS7" s="3" t="inlineStr"/>
+      <c r="AT7" s="3" t="inlineStr"/>
+      <c r="AU7" s="3" t="inlineStr"/>
+      <c r="AV7" s="3" t="inlineStr"/>
+      <c r="AW7" s="3" t="inlineStr">
+        <is>
+          <t>05/2025</t>
+        </is>
+      </c>
+      <c r="AX7" s="3" t="inlineStr">
+        <is>
+          <t>02/2026</t>
+        </is>
+      </c>
+      <c r="AY7" s="3" t="inlineStr"/>
+      <c r="AZ7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>MND-09</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>06/2026</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>DUMMY. Levels = latest old form MND_09.pdf (total 21); MM/YYYY dates invented, onset back-dated to 08/2024. DUMMY. Treatment dates invented. last_assessed = month of the latest old form.</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>11/2025</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr"/>
+      <c r="G8" s="3" t="inlineStr"/>
+      <c r="H8" s="3" t="inlineStr"/>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>06/2025</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr"/>
+      <c r="K8" s="3" t="inlineStr"/>
+      <c r="L8" s="3" t="inlineStr"/>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>09/2024</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>05/2025</t>
+        </is>
+      </c>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="P8" s="3" t="inlineStr"/>
+      <c r="Q8" s="3" t="inlineStr">
+        <is>
+          <t>09/2024</t>
+        </is>
+      </c>
+      <c r="R8" s="3" t="inlineStr"/>
+      <c r="S8" s="3" t="inlineStr"/>
+      <c r="T8" s="3" t="inlineStr"/>
+      <c r="U8" s="3" t="inlineStr">
+        <is>
+          <t>05/2025</t>
+        </is>
+      </c>
+      <c r="V8" s="3" t="inlineStr"/>
+      <c r="W8" s="3" t="inlineStr"/>
+      <c r="X8" s="3" t="inlineStr"/>
+      <c r="Y8" s="3" t="inlineStr">
+        <is>
+          <t>11/2024</t>
+        </is>
+      </c>
+      <c r="Z8" s="3" t="inlineStr">
+        <is>
+          <t>06/2025</t>
+        </is>
+      </c>
+      <c r="AA8" s="3" t="inlineStr">
+        <is>
+          <t>10/2025</t>
+        </is>
+      </c>
+      <c r="AB8" s="3" t="inlineStr"/>
+      <c r="AC8" s="3" t="inlineStr">
+        <is>
+          <t>05/2025</t>
+        </is>
+      </c>
+      <c r="AD8" s="3" t="inlineStr"/>
+      <c r="AE8" s="3" t="inlineStr"/>
+      <c r="AF8" s="3" t="inlineStr"/>
+      <c r="AG8" s="3" t="inlineStr">
+        <is>
+          <t>08/2024</t>
+        </is>
+      </c>
+      <c r="AH8" s="3" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+      <c r="AI8" s="3" t="inlineStr"/>
+      <c r="AJ8" s="3" t="inlineStr"/>
+      <c r="AK8" s="3" t="inlineStr">
+        <is>
+          <t>08/2024</t>
+        </is>
+      </c>
+      <c r="AL8" s="3" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
+      <c r="AM8" s="3" t="inlineStr">
+        <is>
+          <t>07/2025</t>
+        </is>
+      </c>
+      <c r="AN8" s="3" t="inlineStr">
+        <is>
+          <t>12/2025</t>
+        </is>
+      </c>
+      <c r="AO8" s="3" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
+      <c r="AP8" s="3" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+      <c r="AQ8" s="3" t="inlineStr">
+        <is>
+          <t>12/2025</t>
+        </is>
+      </c>
+      <c r="AR8" s="3" t="inlineStr"/>
+      <c r="AS8" s="3" t="inlineStr">
+        <is>
+          <t>09/2024</t>
+        </is>
+      </c>
+      <c r="AT8" s="3" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
+      <c r="AU8" s="3" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+      <c r="AV8" s="3" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="AW8" s="3" t="inlineStr">
+        <is>
+          <t>08/2024</t>
+        </is>
+      </c>
+      <c r="AX8" s="3" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
+      <c r="AY8" s="3" t="inlineStr">
+        <is>
+          <t>09/2025</t>
+        </is>
+      </c>
+      <c r="AZ8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>MND-10</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>06/2026</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>DUMMY. Levels = latest old form MND_10_Jun2026.pdf (total 26); old forms in order: MND_10_26Nov2025.pdf (38), MND_10_05Jan2026.pdf (34), MND_10_Jun2026.pdf (26); MM/YYYY dates invented, onset back-dated to 08/2024; earlier old form scored lower, latest level kept: q4 1→3, q5 2→3. DUMMY. Treatment dates invented. last_assessed = month of the latest old form.</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>08/2024</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr"/>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>06/2025</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr"/>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>10/2024</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>03/2026</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="inlineStr"/>
+      <c r="P9" s="3" t="inlineStr"/>
+      <c r="Q9" s="3" t="inlineStr">
+        <is>
+          <t>06/2025</t>
+        </is>
+      </c>
+      <c r="R9" s="3" t="inlineStr"/>
+      <c r="S9" s="3" t="inlineStr"/>
+      <c r="T9" s="3" t="inlineStr"/>
+      <c r="U9" s="3" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="V9" s="3" t="inlineStr"/>
+      <c r="W9" s="3" t="inlineStr"/>
+      <c r="X9" s="3" t="inlineStr"/>
+      <c r="Y9" s="3" t="inlineStr"/>
+      <c r="Z9" s="3" t="inlineStr"/>
+      <c r="AA9" s="3" t="inlineStr"/>
+      <c r="AB9" s="3" t="inlineStr"/>
+      <c r="AC9" s="3" t="inlineStr"/>
+      <c r="AD9" s="3" t="inlineStr"/>
+      <c r="AE9" s="3" t="inlineStr"/>
+      <c r="AF9" s="3" t="inlineStr"/>
+      <c r="AG9" s="3" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
+      <c r="AH9" s="3" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="AI9" s="3" t="inlineStr"/>
+      <c r="AJ9" s="3" t="inlineStr"/>
+      <c r="AK9" s="3" t="inlineStr">
+        <is>
+          <t>02/2025</t>
+        </is>
+      </c>
+      <c r="AL9" s="3" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="AM9" s="3" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="AN9" s="3" t="inlineStr"/>
+      <c r="AO9" s="3" t="inlineStr">
+        <is>
+          <t>11/2024</t>
+        </is>
+      </c>
+      <c r="AP9" s="3" t="inlineStr">
+        <is>
+          <t>03/2026</t>
+        </is>
+      </c>
+      <c r="AQ9" s="3" t="inlineStr"/>
+      <c r="AR9" s="3" t="inlineStr"/>
+      <c r="AS9" s="3" t="inlineStr">
+        <is>
+          <t>05/2025</t>
+        </is>
+      </c>
+      <c r="AT9" s="3" t="inlineStr">
+        <is>
+          <t>02/2026</t>
+        </is>
+      </c>
+      <c r="AU9" s="3" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="AV9" s="3" t="inlineStr"/>
+      <c r="AW9" s="3" t="inlineStr">
+        <is>
+          <t>03/2026</t>
+        </is>
+      </c>
+      <c r="AX9" s="3" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="AY9" s="3" t="inlineStr"/>
+      <c r="AZ9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>MND-11</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>DUMMY. Levels = latest old form MND_11.pdf (total 46); MM/YYYY dates invented, onset back-dated to 09/2025. DUMMY. Treatment dates invented; no treatment given (test case). last_assessed = month of the latest old form.</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="3" t="inlineStr"/>
+      <c r="G10" s="3" t="inlineStr"/>
+      <c r="H10" s="3" t="inlineStr"/>
+      <c r="I10" s="3" t="inlineStr"/>
+      <c r="J10" s="3" t="inlineStr"/>
+      <c r="K10" s="3" t="inlineStr"/>
+      <c r="L10" s="3" t="inlineStr"/>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>09/2025</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="inlineStr"/>
+      <c r="O10" s="3" t="inlineStr"/>
+      <c r="P10" s="3" t="inlineStr"/>
+      <c r="Q10" s="3" t="inlineStr"/>
+      <c r="R10" s="3" t="inlineStr"/>
+      <c r="S10" s="3" t="inlineStr"/>
+      <c r="T10" s="3" t="inlineStr"/>
+      <c r="U10" s="3" t="inlineStr"/>
+      <c r="V10" s="3" t="inlineStr"/>
+      <c r="W10" s="3" t="inlineStr"/>
+      <c r="X10" s="3" t="inlineStr"/>
+      <c r="Y10" s="3" t="inlineStr"/>
+      <c r="Z10" s="3" t="inlineStr"/>
+      <c r="AA10" s="3" t="inlineStr"/>
+      <c r="AB10" s="3" t="inlineStr"/>
+      <c r="AC10" s="3" t="inlineStr"/>
+      <c r="AD10" s="3" t="inlineStr"/>
+      <c r="AE10" s="3" t="inlineStr"/>
+      <c r="AF10" s="3" t="inlineStr"/>
+      <c r="AG10" s="3" t="inlineStr"/>
+      <c r="AH10" s="3" t="inlineStr"/>
+      <c r="AI10" s="3" t="inlineStr"/>
+      <c r="AJ10" s="3" t="inlineStr"/>
+      <c r="AK10" s="3" t="inlineStr">
+        <is>
+          <t>10/2025</t>
+        </is>
+      </c>
+      <c r="AL10" s="3" t="inlineStr"/>
+      <c r="AM10" s="3" t="inlineStr"/>
+      <c r="AN10" s="3" t="inlineStr"/>
+      <c r="AO10" s="3" t="inlineStr"/>
+      <c r="AP10" s="3" t="inlineStr"/>
+      <c r="AQ10" s="3" t="inlineStr"/>
+      <c r="AR10" s="3" t="inlineStr"/>
+      <c r="AS10" s="3" t="inlineStr"/>
+      <c r="AT10" s="3" t="inlineStr"/>
+      <c r="AU10" s="3" t="inlineStr"/>
+      <c r="AV10" s="3" t="inlineStr"/>
+      <c r="AW10" s="3" t="inlineStr"/>
+      <c r="AX10" s="3" t="inlineStr"/>
+      <c r="AY10" s="3" t="inlineStr"/>
+      <c r="AZ10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>MND-12</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>DUMMY. Levels = latest old form MND_12_15Jan2026.pdf (total 47); old forms in order: MND_12_26Dec2025.pdf (42), MND_12_15Jan2026.pdf (47); MM/YYYY dates invented; earlier old form scored lower, latest level kept: q3 3→4, q4 3→4, q5 3→4, q8 3→4, q9 3→4, q10 3→4. DUMMY. Treatment dates invented; no treatment given (test case). last_assessed = month of the latest old form.</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr"/>
+      <c r="G11" s="3" t="inlineStr"/>
+      <c r="H11" s="3" t="inlineStr"/>
+      <c r="I11" s="3" t="inlineStr"/>
+      <c r="J11" s="3" t="inlineStr"/>
+      <c r="K11" s="3" t="inlineStr"/>
+      <c r="L11" s="3" t="inlineStr"/>
+      <c r="M11" s="3" t="inlineStr"/>
+      <c r="N11" s="3" t="inlineStr"/>
+      <c r="O11" s="3" t="inlineStr"/>
+      <c r="P11" s="3" t="inlineStr"/>
+      <c r="Q11" s="3" t="inlineStr"/>
+      <c r="R11" s="3" t="inlineStr"/>
+      <c r="S11" s="3" t="inlineStr"/>
+      <c r="T11" s="3" t="inlineStr"/>
+      <c r="U11" s="3" t="inlineStr"/>
+      <c r="V11" s="3" t="inlineStr"/>
+      <c r="W11" s="3" t="inlineStr"/>
+      <c r="X11" s="3" t="inlineStr"/>
+      <c r="Y11" s="3" t="inlineStr"/>
+      <c r="Z11" s="3" t="inlineStr"/>
+      <c r="AA11" s="3" t="inlineStr"/>
+      <c r="AB11" s="3" t="inlineStr"/>
+      <c r="AC11" s="3" t="inlineStr"/>
+      <c r="AD11" s="3" t="inlineStr"/>
+      <c r="AE11" s="3" t="inlineStr"/>
+      <c r="AF11" s="3" t="inlineStr"/>
+      <c r="AG11" s="3" t="inlineStr"/>
+      <c r="AH11" s="3" t="inlineStr"/>
+      <c r="AI11" s="3" t="inlineStr"/>
+      <c r="AJ11" s="3" t="inlineStr"/>
+      <c r="AK11" s="3" t="inlineStr"/>
+      <c r="AL11" s="3" t="inlineStr"/>
+      <c r="AM11" s="3" t="inlineStr"/>
+      <c r="AN11" s="3" t="inlineStr"/>
+      <c r="AO11" s="3" t="inlineStr"/>
+      <c r="AP11" s="3" t="inlineStr"/>
+      <c r="AQ11" s="3" t="inlineStr"/>
+      <c r="AR11" s="3" t="inlineStr"/>
+      <c r="AS11" s="3" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="AT11" s="3" t="inlineStr"/>
+      <c r="AU11" s="3" t="inlineStr"/>
+      <c r="AV11" s="3" t="inlineStr"/>
+      <c r="AW11" s="3" t="inlineStr"/>
+      <c r="AX11" s="3" t="inlineStr"/>
+      <c r="AY11" s="3" t="inlineStr"/>
+      <c r="AZ11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>MND-13</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>08/2026</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>DUMMY. Levels = latest old form MND_13_14Aug2026.pdf (total 21); old forms in order: MND_13_16Jan2026.pdf (19), MND_13_14Aug2026.pdf (21); MM/YYYY dates invented, onset back-dated to 02/2024; earlier old form scored lower, latest level kept: q1 1→2, q2 2→4, q5 1→2; test entry: q12 L3 = ?. DUMMY. Treatment dates invented. last_assessed = month of the latest old form.</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>12/2024</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>06/2025</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr"/>
+      <c r="H12" s="3" t="inlineStr"/>
+      <c r="I12" s="3" t="inlineStr"/>
+      <c r="J12" s="3" t="inlineStr"/>
+      <c r="K12" s="3" t="inlineStr"/>
+      <c r="L12" s="3" t="inlineStr"/>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>11/2024</t>
+        </is>
+      </c>
+      <c r="N12" s="3" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
+      <c r="O12" s="3" t="inlineStr"/>
+      <c r="P12" s="3" t="inlineStr"/>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>02/2024</t>
+        </is>
+      </c>
+      <c r="R12" s="3" t="inlineStr">
+        <is>
+          <t>09/2024</t>
+        </is>
+      </c>
+      <c r="S12" s="3" t="inlineStr">
+        <is>
+          <t>06/2025</t>
+        </is>
+      </c>
+      <c r="T12" s="3" t="inlineStr">
+        <is>
+          <t>08/2026</t>
+        </is>
+      </c>
+      <c r="U12" s="3" t="inlineStr">
+        <is>
+          <t>02/2024</t>
+        </is>
+      </c>
+      <c r="V12" s="3" t="inlineStr">
+        <is>
+          <t>12/2024</t>
+        </is>
+      </c>
+      <c r="W12" s="3" t="inlineStr"/>
+      <c r="X12" s="3" t="inlineStr"/>
+      <c r="Y12" s="3" t="inlineStr">
+        <is>
+          <t>04/2024</t>
+        </is>
+      </c>
+      <c r="Z12" s="3" t="inlineStr">
+        <is>
+          <t>12/2024</t>
+        </is>
+      </c>
+      <c r="AA12" s="3" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+      <c r="AB12" s="3" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="AC12" s="3" t="inlineStr">
+        <is>
+          <t>07/2024</t>
+        </is>
+      </c>
+      <c r="AD12" s="3" t="inlineStr">
+        <is>
+          <t>06/2025</t>
+        </is>
+      </c>
+      <c r="AE12" s="3" t="inlineStr"/>
+      <c r="AF12" s="3" t="inlineStr"/>
+      <c r="AG12" s="3" t="inlineStr">
+        <is>
+          <t>09/2024</t>
+        </is>
+      </c>
+      <c r="AH12" s="3" t="inlineStr">
+        <is>
+          <t>02/2025</t>
+        </is>
+      </c>
+      <c r="AI12" s="3" t="inlineStr">
+        <is>
+          <t>09/2025</t>
+        </is>
+      </c>
+      <c r="AJ12" s="3" t="inlineStr"/>
+      <c r="AK12" s="3" t="inlineStr">
+        <is>
+          <t>02/2024</t>
+        </is>
+      </c>
+      <c r="AL12" s="3" t="inlineStr">
+        <is>
+          <t>09/2024</t>
+        </is>
+      </c>
+      <c r="AM12" s="3" t="inlineStr">
+        <is>
+          <t>01/2025</t>
+        </is>
+      </c>
+      <c r="AN12" s="3" t="inlineStr">
+        <is>
+          <t>09/2025</t>
+        </is>
+      </c>
+      <c r="AO12" s="3" t="inlineStr">
+        <is>
+          <t>09/2024</t>
+        </is>
+      </c>
+      <c r="AP12" s="3" t="inlineStr">
+        <is>
+          <t>05/2025</t>
+        </is>
+      </c>
+      <c r="AQ12" s="3" t="inlineStr"/>
+      <c r="AR12" s="3" t="inlineStr"/>
+      <c r="AS12" s="3" t="inlineStr"/>
+      <c r="AT12" s="3" t="inlineStr"/>
+      <c r="AU12" s="3" t="inlineStr"/>
+      <c r="AV12" s="3" t="inlineStr"/>
+      <c r="AW12" s="3" t="inlineStr">
+        <is>
+          <t>09/2024</t>
+        </is>
+      </c>
+      <c r="AX12" s="3" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
+      <c r="AY12" s="3" t="inlineStr"/>
+      <c r="AZ12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>MND-14</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>08/2026</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>DUMMY. Levels = latest old form MND_14.pdf (total 38); MM/YYYY dates invented, onset back-dated to 06/2025. DUMMY. Treatment dates invented. last_assessed = month of the latest old form.</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>02/2026</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr"/>
+      <c r="H13" s="3" t="inlineStr"/>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>11/2025</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr"/>
+      <c r="K13" s="3" t="inlineStr"/>
+      <c r="L13" s="3" t="inlineStr"/>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>02/2026</t>
+        </is>
+      </c>
+      <c r="N13" s="3" t="inlineStr"/>
+      <c r="O13" s="3" t="inlineStr"/>
+      <c r="P13" s="3" t="inlineStr"/>
+      <c r="Q13" s="3" t="inlineStr"/>
+      <c r="R13" s="3" t="inlineStr"/>
+      <c r="S13" s="3" t="inlineStr"/>
+      <c r="T13" s="3" t="inlineStr"/>
+      <c r="U13" s="3" t="inlineStr"/>
+      <c r="V13" s="3" t="inlineStr"/>
+      <c r="W13" s="3" t="inlineStr"/>
+      <c r="X13" s="3" t="inlineStr"/>
+      <c r="Y13" s="3" t="inlineStr"/>
+      <c r="Z13" s="3" t="inlineStr"/>
+      <c r="AA13" s="3" t="inlineStr"/>
+      <c r="AB13" s="3" t="inlineStr"/>
+      <c r="AC13" s="3" t="inlineStr"/>
+      <c r="AD13" s="3" t="inlineStr"/>
+      <c r="AE13" s="3" t="inlineStr"/>
+      <c r="AF13" s="3" t="inlineStr"/>
+      <c r="AG13" s="3" t="inlineStr">
+        <is>
+          <t>07/2025</t>
+        </is>
+      </c>
+      <c r="AH13" s="3" t="inlineStr">
+        <is>
+          <t>03/2026</t>
+        </is>
+      </c>
+      <c r="AI13" s="3" t="inlineStr"/>
+      <c r="AJ13" s="3" t="inlineStr"/>
+      <c r="AK13" s="3" t="inlineStr">
+        <is>
+          <t>06/2025</t>
+        </is>
+      </c>
+      <c r="AL13" s="3" t="inlineStr">
+        <is>
+          <t>10/2025</t>
+        </is>
+      </c>
+      <c r="AM13" s="3" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="AN13" s="3" t="inlineStr"/>
+      <c r="AO13" s="3" t="inlineStr"/>
+      <c r="AP13" s="3" t="inlineStr"/>
+      <c r="AQ13" s="3" t="inlineStr"/>
+      <c r="AR13" s="3" t="inlineStr"/>
+      <c r="AS13" s="3" t="inlineStr"/>
+      <c r="AT13" s="3" t="inlineStr"/>
+      <c r="AU13" s="3" t="inlineStr"/>
+      <c r="AV13" s="3" t="inlineStr"/>
+      <c r="AW13" s="3" t="inlineStr">
+        <is>
+          <t>11/2025</t>
+        </is>
+      </c>
+      <c r="AX13" s="3" t="inlineStr"/>
+      <c r="AY13" s="3" t="inlineStr"/>
+      <c r="AZ13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>MND-15</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>03/2026</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>DUMMY. Levels = latest old form MND_15.pdf (total 30); MM/YYYY dates invented, onset back-dated to 02/2024. DUMMY. Treatment dates invented. last_assessed = month of the latest old form.</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr"/>
+      <c r="F14" s="3" t="inlineStr"/>
+      <c r="G14" s="3" t="inlineStr"/>
+      <c r="H14" s="3" t="inlineStr"/>
+      <c r="I14" s="3" t="inlineStr"/>
+      <c r="J14" s="3" t="inlineStr"/>
+      <c r="K14" s="3" t="inlineStr"/>
+      <c r="L14" s="3" t="inlineStr"/>
+      <c r="M14" s="3" t="inlineStr"/>
+      <c r="N14" s="3" t="inlineStr"/>
+      <c r="O14" s="3" t="inlineStr"/>
+      <c r="P14" s="3" t="inlineStr"/>
+      <c r="Q14" s="3" t="inlineStr">
+        <is>
+          <t>02/2024</t>
+        </is>
+      </c>
+      <c r="R14" s="3" t="inlineStr">
+        <is>
+          <t>08/2024</t>
+        </is>
+      </c>
+      <c r="S14" s="3" t="inlineStr">
+        <is>
+          <t>01/2025</t>
+        </is>
+      </c>
+      <c r="T14" s="3" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+      <c r="U14" s="3" t="inlineStr">
+        <is>
+          <t>02/2024</t>
+        </is>
+      </c>
+      <c r="V14" s="3" t="inlineStr">
+        <is>
+          <t>09/2024</t>
+        </is>
+      </c>
+      <c r="W14" s="3" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
+      <c r="X14" s="3" t="inlineStr">
+        <is>
+          <t>07/2025</t>
+        </is>
+      </c>
+      <c r="Y14" s="3" t="inlineStr">
+        <is>
+          <t>02/2024</t>
+        </is>
+      </c>
+      <c r="Z14" s="3" t="inlineStr">
+        <is>
+          <t>09/2024</t>
+        </is>
+      </c>
+      <c r="AA14" s="3" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
+      <c r="AB14" s="3" t="inlineStr">
+        <is>
+          <t>09/2025</t>
+        </is>
+      </c>
+      <c r="AC14" s="3" t="inlineStr">
+        <is>
+          <t>08/2024</t>
+        </is>
+      </c>
+      <c r="AD14" s="3" t="inlineStr"/>
+      <c r="AE14" s="3" t="inlineStr"/>
+      <c r="AF14" s="3" t="inlineStr"/>
+      <c r="AG14" s="3" t="inlineStr">
+        <is>
+          <t>01/2025</t>
+        </is>
+      </c>
+      <c r="AH14" s="3" t="inlineStr"/>
+      <c r="AI14" s="3" t="inlineStr"/>
+      <c r="AJ14" s="3" t="inlineStr"/>
+      <c r="AK14" s="3" t="inlineStr">
+        <is>
+          <t>05/2024</t>
+        </is>
+      </c>
+      <c r="AL14" s="3" t="inlineStr">
+        <is>
+          <t>09/2024</t>
+        </is>
+      </c>
+      <c r="AM14" s="3" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
+      <c r="AN14" s="3" t="inlineStr">
+        <is>
+          <t>09/2025</t>
+        </is>
+      </c>
+      <c r="AO14" s="3" t="inlineStr"/>
+      <c r="AP14" s="3" t="inlineStr"/>
+      <c r="AQ14" s="3" t="inlineStr"/>
+      <c r="AR14" s="3" t="inlineStr"/>
+      <c r="AS14" s="3" t="inlineStr"/>
+      <c r="AT14" s="3" t="inlineStr"/>
+      <c r="AU14" s="3" t="inlineStr"/>
+      <c r="AV14" s="3" t="inlineStr"/>
+      <c r="AW14" s="3" t="inlineStr"/>
+      <c r="AX14" s="3" t="inlineStr"/>
+      <c r="AY14" s="3" t="inlineStr"/>
+      <c r="AZ14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>MND-16</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>DUMMY. Levels = latest old form MND_16.pdf (total 41); MM/YYYY dates invented, onset back-dated to 03/2025. DUMMY. Treatment dates invented. last_assessed = month of the latest old form.</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr"/>
+      <c r="G15" s="3" t="inlineStr"/>
+      <c r="H15" s="3" t="inlineStr"/>
+      <c r="I15" s="3" t="inlineStr"/>
+      <c r="J15" s="3" t="inlineStr"/>
+      <c r="K15" s="3" t="inlineStr"/>
+      <c r="L15" s="3" t="inlineStr"/>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>09/2025</t>
+        </is>
+      </c>
+      <c r="N15" s="3" t="inlineStr"/>
+      <c r="O15" s="3" t="inlineStr"/>
+      <c r="P15" s="3" t="inlineStr"/>
+      <c r="Q15" s="3" t="inlineStr">
+        <is>
+          <t>10/2025</t>
+        </is>
+      </c>
+      <c r="R15" s="3" t="inlineStr"/>
+      <c r="S15" s="3" t="inlineStr"/>
+      <c r="T15" s="3" t="inlineStr"/>
+      <c r="U15" s="3" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
+      <c r="V15" s="3" t="inlineStr"/>
+      <c r="W15" s="3" t="inlineStr"/>
+      <c r="X15" s="3" t="inlineStr"/>
+      <c r="Y15" s="3" t="inlineStr">
+        <is>
+          <t>05/2025</t>
+        </is>
+      </c>
+      <c r="Z15" s="3" t="inlineStr"/>
+      <c r="AA15" s="3" t="inlineStr"/>
+      <c r="AB15" s="3" t="inlineStr"/>
+      <c r="AC15" s="3" t="inlineStr"/>
+      <c r="AD15" s="3" t="inlineStr"/>
+      <c r="AE15" s="3" t="inlineStr"/>
+      <c r="AF15" s="3" t="inlineStr"/>
+      <c r="AG15" s="3" t="inlineStr">
+        <is>
+          <t>07/2025</t>
+        </is>
+      </c>
+      <c r="AH15" s="3" t="inlineStr"/>
+      <c r="AI15" s="3" t="inlineStr"/>
+      <c r="AJ15" s="3" t="inlineStr"/>
+      <c r="AK15" s="3" t="inlineStr">
+        <is>
+          <t>09/2025</t>
+        </is>
+      </c>
+      <c r="AL15" s="3" t="inlineStr"/>
+      <c r="AM15" s="3" t="inlineStr"/>
+      <c r="AN15" s="3" t="inlineStr"/>
+      <c r="AO15" s="3" t="inlineStr"/>
+      <c r="AP15" s="3" t="inlineStr"/>
+      <c r="AQ15" s="3" t="inlineStr"/>
+      <c r="AR15" s="3" t="inlineStr"/>
+      <c r="AS15" s="3" t="inlineStr"/>
+      <c r="AT15" s="3" t="inlineStr"/>
+      <c r="AU15" s="3" t="inlineStr"/>
+      <c r="AV15" s="3" t="inlineStr"/>
+      <c r="AW15" s="3" t="inlineStr"/>
+      <c r="AX15" s="3" t="inlineStr"/>
+      <c r="AY15" s="3" t="inlineStr"/>
+      <c r="AZ15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>MND-17</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>DUMMY. Levels = latest old form MND_17_05May2026.pdf (total 38); old forms in order: MND_17_04Nov2025.pdf (44), MND_17_03Feb2026.pdf (43), MND_17_05May2026.pdf (38); MM/YYYY dates invented, onset back-dated to 09/2025; earlier old form scored lower, latest level kept: q4 1→4. DUMMY. Treatment dates invented. last_assessed = month of the latest old form.</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr"/>
+      <c r="G16" s="3" t="inlineStr"/>
+      <c r="H16" s="3" t="inlineStr"/>
+      <c r="I16" s="3" t="inlineStr"/>
+      <c r="J16" s="3" t="inlineStr"/>
+      <c r="K16" s="3" t="inlineStr"/>
+      <c r="L16" s="3" t="inlineStr"/>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>02/2026</t>
+        </is>
+      </c>
+      <c r="N16" s="3" t="inlineStr"/>
+      <c r="O16" s="3" t="inlineStr"/>
+      <c r="P16" s="3" t="inlineStr"/>
+      <c r="Q16" s="3" t="inlineStr"/>
+      <c r="R16" s="3" t="inlineStr"/>
+      <c r="S16" s="3" t="inlineStr"/>
+      <c r="T16" s="3" t="inlineStr"/>
+      <c r="U16" s="3" t="inlineStr">
+        <is>
+          <t>09/2025</t>
+        </is>
+      </c>
+      <c r="V16" s="3" t="inlineStr"/>
+      <c r="W16" s="3" t="inlineStr"/>
+      <c r="X16" s="3" t="inlineStr"/>
+      <c r="Y16" s="3" t="inlineStr">
+        <is>
+          <t>03/2026</t>
+        </is>
+      </c>
+      <c r="Z16" s="3" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="AA16" s="3" t="inlineStr"/>
+      <c r="AB16" s="3" t="inlineStr"/>
+      <c r="AC16" s="3" t="inlineStr"/>
+      <c r="AD16" s="3" t="inlineStr"/>
+      <c r="AE16" s="3" t="inlineStr"/>
+      <c r="AF16" s="3" t="inlineStr"/>
+      <c r="AG16" s="3" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="AH16" s="3" t="inlineStr"/>
+      <c r="AI16" s="3" t="inlineStr"/>
+      <c r="AJ16" s="3" t="inlineStr"/>
+      <c r="AK16" s="3" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="AL16" s="3" t="inlineStr"/>
+      <c r="AM16" s="3" t="inlineStr"/>
+      <c r="AN16" s="3" t="inlineStr"/>
+      <c r="AO16" s="3" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="AP16" s="3" t="inlineStr"/>
+      <c r="AQ16" s="3" t="inlineStr"/>
+      <c r="AR16" s="3" t="inlineStr"/>
+      <c r="AS16" s="3" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="AT16" s="3" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="AU16" s="3" t="inlineStr"/>
+      <c r="AV16" s="3" t="inlineStr"/>
+      <c r="AW16" s="3" t="inlineStr"/>
+      <c r="AX16" s="3" t="inlineStr"/>
+      <c r="AY16" s="3" t="inlineStr"/>
+      <c r="AZ16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>MND-18</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>03/2026</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>DUMMY. Levels = latest old form MND_18.pdf (total 42); MM/YYYY dates invented, onset back-dated to 06/2025. DUMMY. Treatment dates invented. last_assessed = month of the latest old form.</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>06/2025</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>10/2025</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr"/>
+      <c r="H17" s="3" t="inlineStr"/>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>10/2025</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr"/>
+      <c r="L17" s="3" t="inlineStr"/>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>09/2025</t>
+        </is>
+      </c>
+      <c r="N17" s="3" t="inlineStr"/>
+      <c r="O17" s="3" t="inlineStr"/>
+      <c r="P17" s="3" t="inlineStr"/>
+      <c r="Q17" s="3" t="inlineStr"/>
+      <c r="R17" s="3" t="inlineStr"/>
+      <c r="S17" s="3" t="inlineStr"/>
+      <c r="T17" s="3" t="inlineStr"/>
+      <c r="U17" s="3" t="inlineStr"/>
+      <c r="V17" s="3" t="inlineStr"/>
+      <c r="W17" s="3" t="inlineStr"/>
+      <c r="X17" s="3" t="inlineStr"/>
+      <c r="Y17" s="3" t="inlineStr"/>
+      <c r="Z17" s="3" t="inlineStr"/>
+      <c r="AA17" s="3" t="inlineStr"/>
+      <c r="AB17" s="3" t="inlineStr"/>
+      <c r="AC17" s="3" t="inlineStr"/>
+      <c r="AD17" s="3" t="inlineStr"/>
+      <c r="AE17" s="3" t="inlineStr"/>
+      <c r="AF17" s="3" t="inlineStr"/>
+      <c r="AG17" s="3" t="inlineStr"/>
+      <c r="AH17" s="3" t="inlineStr"/>
+      <c r="AI17" s="3" t="inlineStr"/>
+      <c r="AJ17" s="3" t="inlineStr"/>
+      <c r="AK17" s="3" t="inlineStr"/>
+      <c r="AL17" s="3" t="inlineStr"/>
+      <c r="AM17" s="3" t="inlineStr"/>
+      <c r="AN17" s="3" t="inlineStr"/>
+      <c r="AO17" s="3" t="inlineStr"/>
+      <c r="AP17" s="3" t="inlineStr"/>
+      <c r="AQ17" s="3" t="inlineStr"/>
+      <c r="AR17" s="3" t="inlineStr"/>
+      <c r="AS17" s="3" t="inlineStr">
+        <is>
+          <t>11/2025</t>
+        </is>
+      </c>
+      <c r="AT17" s="3" t="inlineStr"/>
+      <c r="AU17" s="3" t="inlineStr"/>
+      <c r="AV17" s="3" t="inlineStr"/>
+      <c r="AW17" s="3" t="inlineStr"/>
+      <c r="AX17" s="3" t="inlineStr"/>
+      <c r="AY17" s="3" t="inlineStr"/>
+      <c r="AZ17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>MND-19</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>DUMMY. Levels = latest old form MND_19.pdf (total 13); MM/YYYY dates invented, onset back-dated to 06/2023; test entry: q8 L3 = 2023. DUMMY. Treatment dates invented. last_assessed = month of the latest old form.</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>06/2023</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>02/2024</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>11/2024</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>11/2023</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>08/2024</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>01/2025</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>07/2025</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>06/2024</t>
+        </is>
+      </c>
+      <c r="N18" s="3" t="inlineStr">
+        <is>
+          <t>05/2025</t>
+        </is>
+      </c>
+      <c r="O18" s="3" t="inlineStr"/>
+      <c r="P18" s="3" t="inlineStr"/>
+      <c r="Q18" s="3" t="inlineStr">
+        <is>
+          <t>08/2023</t>
+        </is>
+      </c>
+      <c r="R18" s="3" t="inlineStr">
+        <is>
+          <t>05/2024</t>
+        </is>
+      </c>
+      <c r="S18" s="3" t="inlineStr">
+        <is>
+          <t>11/2024</t>
+        </is>
+      </c>
+      <c r="T18" s="3" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+      <c r="U18" s="3" t="inlineStr">
+        <is>
+          <t>08/2023</t>
+        </is>
+      </c>
+      <c r="V18" s="3" t="inlineStr">
+        <is>
+          <t>02/2024</t>
+        </is>
+      </c>
+      <c r="W18" s="3" t="inlineStr">
+        <is>
+          <t>10/2024</t>
+        </is>
+      </c>
+      <c r="X18" s="3" t="inlineStr">
+        <is>
+          <t>07/2025</t>
+        </is>
+      </c>
+      <c r="Y18" s="3" t="inlineStr">
+        <is>
+          <t>12/2023</t>
+        </is>
+      </c>
+      <c r="Z18" s="3" t="inlineStr">
+        <is>
+          <t>08/2024</t>
+        </is>
+      </c>
+      <c r="AA18" s="3" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+      <c r="AB18" s="3" t="inlineStr"/>
+      <c r="AC18" s="3" t="inlineStr">
+        <is>
+          <t>07/2023</t>
+        </is>
+      </c>
+      <c r="AD18" s="3" t="inlineStr">
+        <is>
+          <t>03/2024</t>
+        </is>
+      </c>
+      <c r="AE18" s="3" t="inlineStr">
+        <is>
+          <t>11/2024</t>
+        </is>
+      </c>
+      <c r="AF18" s="3" t="inlineStr">
+        <is>
+          <t>05/2025</t>
+        </is>
+      </c>
+      <c r="AG18" s="3" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="AH18" s="3" t="inlineStr">
+        <is>
+          <t>02/2024</t>
+        </is>
+      </c>
+      <c r="AI18" s="3" t="inlineStr">
+        <is>
+          <t>11/2024</t>
+        </is>
+      </c>
+      <c r="AJ18" s="3" t="inlineStr">
+        <is>
+          <t>05/2025</t>
+        </is>
+      </c>
+      <c r="AK18" s="3" t="inlineStr">
+        <is>
+          <t>07/2023</t>
+        </is>
+      </c>
+      <c r="AL18" s="3" t="inlineStr">
+        <is>
+          <t>02/2024</t>
+        </is>
+      </c>
+      <c r="AM18" s="3" t="inlineStr">
+        <is>
+          <t>01/2025</t>
+        </is>
+      </c>
+      <c r="AN18" s="3" t="inlineStr">
+        <is>
+          <t>07/2025</t>
+        </is>
+      </c>
+      <c r="AO18" s="3" t="inlineStr">
+        <is>
+          <t>10/2024</t>
+        </is>
+      </c>
+      <c r="AP18" s="3" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+      <c r="AQ18" s="3" t="inlineStr"/>
+      <c r="AR18" s="3" t="inlineStr"/>
+      <c r="AS18" s="3" t="inlineStr"/>
+      <c r="AT18" s="3" t="inlineStr"/>
+      <c r="AU18" s="3" t="inlineStr"/>
+      <c r="AV18" s="3" t="inlineStr"/>
+      <c r="AW18" s="3" t="inlineStr"/>
+      <c r="AX18" s="3" t="inlineStr"/>
+      <c r="AY18" s="3" t="inlineStr"/>
+      <c r="AZ18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>MND-20</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>DUMMY. Levels = latest old form MND_20.pdf (total 30); MM/YYYY dates invented, onset back-dated to 07/2024. DUMMY. Treatment dates invented. last_assessed = month of the latest old form.</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>10/2025</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr"/>
+      <c r="H19" s="3" t="inlineStr"/>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>02/2025</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>09/2025</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr"/>
+      <c r="L19" s="3" t="inlineStr"/>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>06/2025</t>
+        </is>
+      </c>
+      <c r="N19" s="3" t="inlineStr">
+        <is>
+          <t>11/2025</t>
+        </is>
+      </c>
+      <c r="O19" s="3" t="inlineStr"/>
+      <c r="P19" s="3" t="inlineStr"/>
+      <c r="Q19" s="3" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
+      <c r="R19" s="3" t="inlineStr"/>
+      <c r="S19" s="3" t="inlineStr"/>
+      <c r="T19" s="3" t="inlineStr"/>
+      <c r="U19" s="3" t="inlineStr">
+        <is>
+          <t>08/2024</t>
+        </is>
+      </c>
+      <c r="V19" s="3" t="inlineStr">
+        <is>
+          <t>09/2025</t>
+        </is>
+      </c>
+      <c r="W19" s="3" t="inlineStr"/>
+      <c r="X19" s="3" t="inlineStr"/>
+      <c r="Y19" s="3" t="inlineStr">
+        <is>
+          <t>08/2024</t>
+        </is>
+      </c>
+      <c r="Z19" s="3" t="inlineStr"/>
+      <c r="AA19" s="3" t="inlineStr"/>
+      <c r="AB19" s="3" t="inlineStr"/>
+      <c r="AC19" s="3" t="inlineStr"/>
+      <c r="AD19" s="3" t="inlineStr"/>
+      <c r="AE19" s="3" t="inlineStr"/>
+      <c r="AF19" s="3" t="inlineStr"/>
+      <c r="AG19" s="3" t="inlineStr">
+        <is>
+          <t>02/2025</t>
+        </is>
+      </c>
+      <c r="AH19" s="3" t="inlineStr"/>
+      <c r="AI19" s="3" t="inlineStr"/>
+      <c r="AJ19" s="3" t="inlineStr"/>
+      <c r="AK19" s="3" t="inlineStr">
+        <is>
+          <t>07/2024</t>
+        </is>
+      </c>
+      <c r="AL19" s="3" t="inlineStr">
+        <is>
+          <t>12/2024</t>
+        </is>
+      </c>
+      <c r="AM19" s="3" t="inlineStr">
+        <is>
+          <t>05/2025</t>
+        </is>
+      </c>
+      <c r="AN19" s="3" t="inlineStr">
+        <is>
+          <t>11/2025</t>
+        </is>
+      </c>
+      <c r="AO19" s="3" t="inlineStr">
+        <is>
+          <t>11/2024</t>
+        </is>
+      </c>
+      <c r="AP19" s="3" t="inlineStr"/>
+      <c r="AQ19" s="3" t="inlineStr"/>
+      <c r="AR19" s="3" t="inlineStr"/>
+      <c r="AS19" s="3" t="inlineStr">
+        <is>
+          <t>10/2024</t>
+        </is>
+      </c>
+      <c r="AT19" s="3" t="inlineStr">
+        <is>
+          <t>06/2025</t>
+        </is>
+      </c>
+      <c r="AU19" s="3" t="inlineStr"/>
+      <c r="AV19" s="3" t="inlineStr"/>
+      <c r="AW19" s="3" t="inlineStr"/>
+      <c r="AX19" s="3" t="inlineStr"/>
+      <c r="AY19" s="3" t="inlineStr"/>
+      <c r="AZ19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>MND-21</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>DUMMY. Levels = latest old form MND_21.pdf (total 38); MM/YYYY dates invented, onset back-dated to 05/2025. DUMMY. Treatment dates invented. last_assessed = month of the latest old form.</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="3" t="inlineStr"/>
+      <c r="G20" s="3" t="inlineStr"/>
+      <c r="H20" s="3" t="inlineStr"/>
+      <c r="I20" s="3" t="inlineStr"/>
+      <c r="J20" s="3" t="inlineStr"/>
+      <c r="K20" s="3" t="inlineStr"/>
+      <c r="L20" s="3" t="inlineStr"/>
+      <c r="M20" s="3" t="inlineStr"/>
+      <c r="N20" s="3" t="inlineStr"/>
+      <c r="O20" s="3" t="inlineStr"/>
+      <c r="P20" s="3" t="inlineStr"/>
+      <c r="Q20" s="3" t="inlineStr"/>
+      <c r="R20" s="3" t="inlineStr"/>
+      <c r="S20" s="3" t="inlineStr"/>
+      <c r="T20" s="3" t="inlineStr"/>
+      <c r="U20" s="3" t="inlineStr"/>
+      <c r="V20" s="3" t="inlineStr"/>
+      <c r="W20" s="3" t="inlineStr"/>
+      <c r="X20" s="3" t="inlineStr"/>
+      <c r="Y20" s="3" t="inlineStr">
+        <is>
+          <t>06/2025</t>
+        </is>
+      </c>
+      <c r="Z20" s="3" t="inlineStr"/>
+      <c r="AA20" s="3" t="inlineStr"/>
+      <c r="AB20" s="3" t="inlineStr"/>
+      <c r="AC20" s="3" t="inlineStr">
+        <is>
+          <t>07/2025</t>
+        </is>
+      </c>
+      <c r="AD20" s="3" t="inlineStr">
+        <is>
+          <t>12/2025</t>
+        </is>
+      </c>
+      <c r="AE20" s="3" t="inlineStr"/>
+      <c r="AF20" s="3" t="inlineStr"/>
+      <c r="AG20" s="3" t="inlineStr">
+        <is>
+          <t>06/2025</t>
+        </is>
+      </c>
+      <c r="AH20" s="3" t="inlineStr">
+        <is>
+          <t>12/2025</t>
+        </is>
+      </c>
+      <c r="AI20" s="3" t="inlineStr"/>
+      <c r="AJ20" s="3" t="inlineStr"/>
+      <c r="AK20" s="3" t="inlineStr">
+        <is>
+          <t>05/2025</t>
+        </is>
+      </c>
+      <c r="AL20" s="3" t="inlineStr">
+        <is>
+          <t>07/2025</t>
+        </is>
+      </c>
+      <c r="AM20" s="3" t="inlineStr">
+        <is>
+          <t>11/2025</t>
+        </is>
+      </c>
+      <c r="AN20" s="3" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="AO20" s="3" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+      <c r="AP20" s="3" t="inlineStr"/>
+      <c r="AQ20" s="3" t="inlineStr"/>
+      <c r="AR20" s="3" t="inlineStr"/>
+      <c r="AS20" s="3" t="inlineStr"/>
+      <c r="AT20" s="3" t="inlineStr"/>
+      <c r="AU20" s="3" t="inlineStr"/>
+      <c r="AV20" s="3" t="inlineStr"/>
+      <c r="AW20" s="3" t="inlineStr"/>
+      <c r="AX20" s="3" t="inlineStr"/>
+      <c r="AY20" s="3" t="inlineStr"/>
+      <c r="AZ20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>MND-23</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>08/2026</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>DUMMY. Levels = latest old form MND_23_2.pdf (total 46); old forms in order: MND_23_17May2026.pdf (47), MND_23_2.pdf (46); MM/YYYY dates invented, onset back-dated to 03/2026; old form undated, assessment month assumed 08/2026. DUMMY. Treatment dates invented. last_assessed = month of the latest old form (assumed, old form undated).</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr"/>
+      <c r="G21" s="3" t="inlineStr"/>
+      <c r="H21" s="3" t="inlineStr"/>
+      <c r="I21" s="3" t="inlineStr"/>
+      <c r="J21" s="3" t="inlineStr"/>
+      <c r="K21" s="3" t="inlineStr"/>
+      <c r="L21" s="3" t="inlineStr"/>
+      <c r="M21" s="3" t="inlineStr"/>
+      <c r="N21" s="3" t="inlineStr"/>
+      <c r="O21" s="3" t="inlineStr"/>
+      <c r="P21" s="3" t="inlineStr"/>
+      <c r="Q21" s="3" t="inlineStr">
+        <is>
+          <t>03/2026</t>
+        </is>
+      </c>
+      <c r="R21" s="3" t="inlineStr"/>
+      <c r="S21" s="3" t="inlineStr"/>
+      <c r="T21" s="3" t="inlineStr"/>
+      <c r="U21" s="3" t="inlineStr">
+        <is>
+          <t>06/2026</t>
+        </is>
+      </c>
+      <c r="V21" s="3" t="inlineStr"/>
+      <c r="W21" s="3" t="inlineStr"/>
+      <c r="X21" s="3" t="inlineStr"/>
+      <c r="Y21" s="3" t="inlineStr"/>
+      <c r="Z21" s="3" t="inlineStr"/>
+      <c r="AA21" s="3" t="inlineStr"/>
+      <c r="AB21" s="3" t="inlineStr"/>
+      <c r="AC21" s="3" t="inlineStr"/>
+      <c r="AD21" s="3" t="inlineStr"/>
+      <c r="AE21" s="3" t="inlineStr"/>
+      <c r="AF21" s="3" t="inlineStr"/>
+      <c r="AG21" s="3" t="inlineStr"/>
+      <c r="AH21" s="3" t="inlineStr"/>
+      <c r="AI21" s="3" t="inlineStr"/>
+      <c r="AJ21" s="3" t="inlineStr"/>
+      <c r="AK21" s="3" t="inlineStr"/>
+      <c r="AL21" s="3" t="inlineStr"/>
+      <c r="AM21" s="3" t="inlineStr"/>
+      <c r="AN21" s="3" t="inlineStr"/>
+      <c r="AO21" s="3" t="inlineStr"/>
+      <c r="AP21" s="3" t="inlineStr"/>
+      <c r="AQ21" s="3" t="inlineStr"/>
+      <c r="AR21" s="3" t="inlineStr"/>
+      <c r="AS21" s="3" t="inlineStr"/>
+      <c r="AT21" s="3" t="inlineStr"/>
+      <c r="AU21" s="3" t="inlineStr"/>
+      <c r="AV21" s="3" t="inlineStr"/>
+      <c r="AW21" s="3" t="inlineStr"/>
+      <c r="AX21" s="3" t="inlineStr"/>
+      <c r="AY21" s="3" t="inlineStr"/>
+      <c r="AZ21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>MND-24</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>06/2026</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>DUMMY. Levels = latest old form MND_24.pdf (total 24); MM/YYYY dates invented, onset back-dated to 11/2024; test entry: q7 L3 = 2025. DUMMY. Treatment dates invented. last_assessed = month of the latest old form.</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>02/2026</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr"/>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>05/2025</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>11/2025</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr"/>
+      <c r="L22" s="3" t="inlineStr"/>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>09/2025</t>
+        </is>
+      </c>
+      <c r="N22" s="3" t="inlineStr">
+        <is>
+          <t>03/2026</t>
+        </is>
+      </c>
+      <c r="O22" s="3" t="inlineStr"/>
+      <c r="P22" s="3" t="inlineStr"/>
+      <c r="Q22" s="3" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
+      <c r="R22" s="3" t="inlineStr">
+        <is>
+          <t>12/2025</t>
+        </is>
+      </c>
+      <c r="S22" s="3" t="inlineStr"/>
+      <c r="T22" s="3" t="inlineStr"/>
+      <c r="U22" s="3" t="inlineStr">
+        <is>
+          <t>12/2024</t>
+        </is>
+      </c>
+      <c r="V22" s="3" t="inlineStr">
+        <is>
+          <t>05/2025</t>
+        </is>
+      </c>
+      <c r="W22" s="3" t="inlineStr">
+        <is>
+          <t>11/2025</t>
+        </is>
+      </c>
+      <c r="X22" s="3" t="inlineStr"/>
+      <c r="Y22" s="3" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
+      <c r="Z22" s="3" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+      <c r="AA22" s="3" t="inlineStr">
+        <is>
+          <t>02/2026</t>
+        </is>
+      </c>
+      <c r="AB22" s="3" t="inlineStr"/>
+      <c r="AC22" s="3" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="AD22" s="3" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+      <c r="AE22" s="3" t="inlineStr">
+        <is>
+          <t>12/2025</t>
+        </is>
+      </c>
+      <c r="AF22" s="3" t="inlineStr"/>
+      <c r="AG22" s="3" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
+      <c r="AH22" s="3" t="inlineStr">
+        <is>
+          <t>11/2025</t>
+        </is>
+      </c>
+      <c r="AI22" s="3" t="inlineStr"/>
+      <c r="AJ22" s="3" t="inlineStr"/>
+      <c r="AK22" s="3" t="inlineStr">
+        <is>
+          <t>11/2024</t>
+        </is>
+      </c>
+      <c r="AL22" s="3" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
+      <c r="AM22" s="3" t="inlineStr">
+        <is>
+          <t>07/2025</t>
+        </is>
+      </c>
+      <c r="AN22" s="3" t="inlineStr">
+        <is>
+          <t>03/2026</t>
+        </is>
+      </c>
+      <c r="AO22" s="3" t="inlineStr"/>
+      <c r="AP22" s="3" t="inlineStr"/>
+      <c r="AQ22" s="3" t="inlineStr"/>
+      <c r="AR22" s="3" t="inlineStr"/>
+      <c r="AS22" s="3" t="inlineStr"/>
+      <c r="AT22" s="3" t="inlineStr"/>
+      <c r="AU22" s="3" t="inlineStr"/>
+      <c r="AV22" s="3" t="inlineStr"/>
+      <c r="AW22" s="3" t="inlineStr"/>
+      <c r="AX22" s="3" t="inlineStr"/>
+      <c r="AY22" s="3" t="inlineStr"/>
+      <c r="AZ22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>MND-25</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>09/2026</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>DUMMY. Levels = latest old form MND_25.pdf (total 44); MM/YYYY dates invented, onset back-dated to 02/2026; old form undated, assessment month assumed 09/2026. DUMMY. Treatment dates invented. last_assessed = month of the latest old form (assumed, old form undated).</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr"/>
+      <c r="G23" s="3" t="inlineStr"/>
+      <c r="H23" s="3" t="inlineStr"/>
+      <c r="I23" s="3" t="inlineStr"/>
+      <c r="J23" s="3" t="inlineStr"/>
+      <c r="K23" s="3" t="inlineStr"/>
+      <c r="L23" s="3" t="inlineStr"/>
+      <c r="M23" s="3" t="inlineStr"/>
+      <c r="N23" s="3" t="inlineStr"/>
+      <c r="O23" s="3" t="inlineStr"/>
+      <c r="P23" s="3" t="inlineStr"/>
+      <c r="Q23" s="3" t="inlineStr"/>
+      <c r="R23" s="3" t="inlineStr"/>
+      <c r="S23" s="3" t="inlineStr"/>
+      <c r="T23" s="3" t="inlineStr"/>
+      <c r="U23" s="3" t="inlineStr"/>
+      <c r="V23" s="3" t="inlineStr"/>
+      <c r="W23" s="3" t="inlineStr"/>
+      <c r="X23" s="3" t="inlineStr"/>
+      <c r="Y23" s="3" t="inlineStr"/>
+      <c r="Z23" s="3" t="inlineStr"/>
+      <c r="AA23" s="3" t="inlineStr"/>
+      <c r="AB23" s="3" t="inlineStr"/>
+      <c r="AC23" s="3" t="inlineStr">
+        <is>
+          <t>02/2026</t>
+        </is>
+      </c>
+      <c r="AD23" s="3" t="inlineStr"/>
+      <c r="AE23" s="3" t="inlineStr"/>
+      <c r="AF23" s="3" t="inlineStr"/>
+      <c r="AG23" s="3" t="inlineStr">
+        <is>
+          <t>02/2026</t>
+        </is>
+      </c>
+      <c r="AH23" s="3" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="AI23" s="3" t="inlineStr"/>
+      <c r="AJ23" s="3" t="inlineStr"/>
+      <c r="AK23" s="3" t="inlineStr">
+        <is>
+          <t>03/2026</t>
+        </is>
+      </c>
+      <c r="AL23" s="3" t="inlineStr"/>
+      <c r="AM23" s="3" t="inlineStr"/>
+      <c r="AN23" s="3" t="inlineStr"/>
+      <c r="AO23" s="3" t="inlineStr"/>
+      <c r="AP23" s="3" t="inlineStr"/>
+      <c r="AQ23" s="3" t="inlineStr"/>
+      <c r="AR23" s="3" t="inlineStr"/>
+      <c r="AS23" s="3" t="inlineStr"/>
+      <c r="AT23" s="3" t="inlineStr"/>
+      <c r="AU23" s="3" t="inlineStr"/>
+      <c r="AV23" s="3" t="inlineStr"/>
+      <c r="AW23" s="3" t="inlineStr"/>
+      <c r="AX23" s="3" t="inlineStr"/>
+      <c r="AY23" s="3" t="inlineStr"/>
+      <c r="AZ23" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="B2:B2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="TH or EN" type="list" errorStyle="warning">
@@ -918,7 +3634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="3" min="1" max="1"/>
@@ -954,6 +3670,527 @@
           <t>notes</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>MND-02</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Riluzole</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>12/2025</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>MND-04</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Riluzole</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>11/2025</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>MND-05</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Riluzole</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>10/2025</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>MND-06</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Riluzole</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>03/2026</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>MND-07</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Riluzole</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>11/2025</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>MND-07</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Edaravone</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>03/2026</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>MND-08</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Riluzole</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>06/2025</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>MND-08</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Edaravone</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>11/2025</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>MND-09</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Riluzole</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>08/2025</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>MND-09</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Edaravone</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>11/2025</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>MND-10</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Riluzole</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>07/2025</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>MND-10</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Edaravone</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>12/2025</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>MND-13</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Riluzole</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>01/2025</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>MND-13</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Edaravone</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>06/2025</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>MND-14</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Riluzole</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>12/2025</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>MND-15</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Riluzole</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>MND-16</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Riluzole</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>09/2025</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>MND-17</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Riluzole</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>MND-18</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Riluzole</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>11/2025</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>MND-19</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Riluzole</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>10/2024</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>MND-19</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Edaravone</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>12/2024</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>07/2025</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>MND-20</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Riluzole</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>06/2025</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>MND-21</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Riluzole</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>11/2025</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>MND-23</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Riluzole</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>06/2026</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>MND-24</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Riluzole</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>06/2025</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>MND-24</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Edaravone</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>11/2025</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>MND-25</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Riluzole</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="4">

</xml_diff>